<commit_message>
fix(data): correct all 112 broken image URLs (remove _item.png suffix)
API scraper appended '_item.png' to every CDN filename, producing broken
URLs like 'sunomono_item.png' instead of 'sunomono.jpg'. Fixed by using
DOM-scraped URLs (original .jpg/.webp) where available (99 items) and
stripping the '_item.png' suffix for the remaining 13 items.

Regenerated sushi-cazza-cardapio.xlsx and public/sushi-cazza-cardapio.xlsx
with corrected image URLs.

https://claude.ai/code/session_01TxV6o1iktVrYiGm8JqoQJ1
</commit_message>
<xml_diff>
--- a/data/sushi-cazza-cardapio.xlsx
+++ b/data/sushi-cazza-cardapio.xlsx
@@ -446,7 +446,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2710303/photo1756325207.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2710303/photo1756325207.jpeg</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -471,7 +471,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970292/photo1724225413.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970292/photo1724225413.jpeg.webp</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -496,7 +496,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970279/325125_original_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970279/325125_original.jpg</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -521,7 +521,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970280/c9996acd834cbeaf810bc257183b72a7_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970280/c9996acd834cbeaf810bc257183b72a7.jpg</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -546,7 +546,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970283/sunomono_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970283/sunomono.jpg</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -571,7 +571,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970281/SHIMEJI_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970281/SHIMEJI.jpg</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -596,7 +596,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970286/68bf0ef705a832e831c27dc5083235f5_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970286/68bf0ef705a832e831c27dc5083235f5.jpg</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -616,7 +616,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970285/HARUMAKI_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970285/HARUMAKI.jpg</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -641,7 +641,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2551663/photo1732344546.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2551663/photo1732344546.jpeg.webp</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970751/photo1724224627.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970751/photo1724224627.jpeg.webp</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -691,7 +691,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970752/ifood_38_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970752/ifood_38.jpg</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -716,7 +716,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970442/photo1724224710.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970442/photo1724224710.jpeg.webp</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -741,7 +741,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970441/photo1724224834.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970441/photo1724224834.jpeg.webp</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -766,7 +766,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2504179/photo1726637627.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2504179/photo1726637627.jpeg.webp</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -791,7 +791,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2504178/photo1726637522.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2504178/photo1726637522.jpeg.webp</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -816,7 +816,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970748/photo1724224670.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970748/photo1724224670.jpeg.webp</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -841,7 +841,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970756/photo1724224527.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970756/photo1724224527.jpeg.webp</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -866,7 +866,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970754/photo1724224582.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970754/photo1724224582.jpeg.webp</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -891,7 +891,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970303/photo1726638153.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970303/photo1726638153.jpeg.webp</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -916,7 +916,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970384/photo1724224922.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970384/photo1724224922.jpeg.webp</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -936,7 +936,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970382/photo1724224960.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970382/photo1724224960.jpeg.webp</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -961,7 +961,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970380/photo1724225023.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970380/photo1724225023.jpeg.webp</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -986,7 +986,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970377/photo1724225082.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970377/photo1724225082.jpeg.webp</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1011,7 +1011,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2637650/photo1756207676.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2637650/photo1756207676.jpeg.webp</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1036,7 +1036,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2351451/photo1724224389.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2351451/photo1724224389.jpeg.webp</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1061,7 +1061,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483441/photo1724222384.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483441/photo1724222384.jpeg.webp</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1086,7 +1086,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2433692/photo1720111023.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2433692/photo1720111023.jpeg.webp</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1111,7 +1111,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2551668/photo1732349913.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2551668/photo1732349913.jpeg.webp</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1136,7 +1136,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2551667/photo1732349754.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2551667/photo1732349754.jpeg.webp</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1161,7 +1161,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2504173/photo1732342042.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2504173/photo1732342042.jpeg.webp</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1186,7 +1186,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2504172/photo1726757055.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2504172/photo1726757055.jpeg.webp</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1211,7 +1211,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2504171/photo1726757108.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2504171/photo1726757108.jpeg.webp</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1236,7 +1236,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2504170/photo1726757137.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2504170/photo1726757137.jpeg.webp</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1261,7 +1261,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2695512/photo1756187706.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2695512/photo1756187706.jpeg.webp</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1286,7 +1286,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2695511/photo1756207404.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2695511/photo1756207404.jpeg.webp</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1311,7 +1311,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2695497/photo1756207720.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2695497/photo1756207720.jpeg.webp</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1336,7 +1336,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970296/WhatsApp_Image_2021-05-19_at_14.28.21__2__item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970296/WhatsApp_Image_2021-05-19_at_14.28.21__2_.jpeg</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1361,7 +1361,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483468/WhatsApp_Image_2021-05-19_at_14_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483468/WhatsApp_Image_2021-05-19_at_14.webp</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1386,7 +1386,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2438265/photo1724222424.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2438265/photo1724222424.jpeg</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1411,7 +1411,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483458/WhatsApp_Image_2021-05-19_at_14_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483458/WhatsApp_Image_2021-05-19_at_14.webp</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1436,7 +1436,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483486/photo1709854584.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483486/photo1709854584.jpeg.webp</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1461,7 +1461,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2303064/photo1709854709.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2303064/photo1709854709.jpeg.webp</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1486,7 +1486,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2364982/photo1713996122.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2364982/photo1713996122.jpeg.webp</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1511,7 +1511,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483445/ifood_50_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483445/ifood_50.webp</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1536,7 +1536,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970428/ifood_50_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970428/ifood_50.jpg</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1561,7 +1561,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2551669/photo1732350463.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2551669/photo1732350463.jpeg.webp</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1586,7 +1586,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970427/download__7__item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970427/download__7_.jpg</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1611,7 +1611,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483474/photo1704404283.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483474/photo1704404283.jpeg.webp</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1636,7 +1636,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483473/photo1704404228.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483473/photo1704404228.jpeg.webp</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1661,7 +1661,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2551673/photo1732350879.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2551673/photo1732350879.jpeg.webp</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1686,7 +1686,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2551674/photo1732351002.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2551674/photo1732351002.jpeg.webp</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1711,7 +1711,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2770750/photo1772587458.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2770750/photo1772587458.jpeg.webp</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1736,7 +1736,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2710906/photo1756356069.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2710906/photo1756356069.jpeg.webp</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1761,7 +1761,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483483/photo1678900166.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483483/photo1678900166.jpeg.webp</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1786,7 +1786,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483477/photo1756350773.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483477/photo1756350773.jpeg.webp</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1811,7 +1811,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2711095/photo1756430337.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2711095/photo1756430337.jpeg.webp</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1836,7 +1836,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970350/ifood_95_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970350/ifood_95.jpg</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1861,7 +1861,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2551665/photo1732347711.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2551665/photo1732347711.jpeg.webp</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1886,7 +1886,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970349/download__5__item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970349/download__5_.jpg</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1911,7 +1911,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970341/photo1724225345.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970341/photo1724225345.jpeg.webp</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1936,7 +1936,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970343/photo1724225304.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970343/photo1724225304.jpeg.webp</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1961,7 +1961,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2504177/photo1726637332.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2504177/photo1726637332.jpeg.webp</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1986,7 +1986,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2351452/photo1712960053.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2351452/photo1712960053.jpeg.webp</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2011,7 +2011,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970348/5efe07ad-6dc8-4cad-b60c-2a9aac1e01b4_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970348/5efe07ad-6dc8-4cad-b60c-2a9aac1e01b4.jpg</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2036,7 +2036,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2551664/photo1732347601.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2551664/photo1732347601.jpeg.webp</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2061,7 +2061,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2551666/photo1732348661.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2551666/photo1732348661.jpeg.webp</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2086,7 +2086,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2504181/photo1731547418.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2504181/photo1731547418.jpeg.webp</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2111,7 +2111,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2504176/photo1726637063.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2504176/photo1726637063.jpeg.webp</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2136,7 +2136,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483449/ifood_1__1__item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483449/ifood_1__1_.webp</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2161,7 +2161,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483448/download__3__item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483448/download__3_.webp</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2186,7 +2186,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970324/264a7a68-2ed7-4b07-81fd-50958a8836fe-1611320198005_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970324/264a7a68-2ed7-4b07-81fd-50958a8836fe-1611320198005.png</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2211,7 +2211,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970353/photo1724225202.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970353/photo1724225202.jpeg.webp</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2236,7 +2236,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970352/photo1724225257.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970352/photo1724225257.jpeg.webp</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2261,7 +2261,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483451/ifood_12_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483451/ifood_12.webp</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2286,7 +2286,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483450/WhatsApp_Image_2021-05-19_at_14_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483450/WhatsApp_Image_2021-05-19_at_14.webp</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2311,7 +2311,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483452/photo1712803347.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483452/photo1712803347.jpeg.webp</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2336,7 +2336,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483466/ifood_18_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483466/ifood_18.webp</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2361,7 +2361,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483463/images_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483463/images.webp</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2386,7 +2386,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483462/WhatsApp_Image_2021-05-19_at_14_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483462/WhatsApp_Image_2021-05-19_at_14.webp</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2411,7 +2411,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483467/Uramaki_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483467/Uramaki.webp</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2436,7 +2436,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2551662/photo1732342823.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2551662/photo1732342823.jpeg.webp</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2461,7 +2461,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483461/sushi-hokkai_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483461/sushi-hokkai.webp</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2486,7 +2486,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2436773/photo1720111994.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2436773/photo1720111994.jpeg.webp</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2511,7 +2511,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970316/download__1__item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970316/download__1_.jpg</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2536,7 +2536,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970315/WhatsApp_Image_2021-05-19_at_14.28.21__4__item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970315/WhatsApp_Image_2021-05-19_at_14.28.21__4_.jpeg</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2561,7 +2561,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2486770/photo1724816650.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2486770/photo1724816650.jpeg</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2586,7 +2586,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2486768/photo1756208261.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2486768/photo1756208261.jpeg</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2611,7 +2611,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2486767/photo1724816049.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2486767/photo1724816049.jpeg</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2636,7 +2636,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2486766/photo1756208324.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2486766/photo1756208324.jpeg</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2661,7 +2661,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2770743/photo1772583500.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2770743/photo1772583500.jpeg.webp</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2686,7 +2686,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970902/Agua_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970902/Agua.jpg</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2706,7 +2706,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/970900/Agua-c-g_s_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/970900/Agua-c-g_s.jpg</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2726,7 +2726,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2436286/photo1720103827.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2436286/photo1720103827.jpeg.webp</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2751,7 +2751,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2436761/photo1720109634.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2436761/photo1720109634.jpeg</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2771,7 +2771,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2486771/photo1724817008.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2486771/photo1724817008.jpeg</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2796,7 +2796,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2436769/photo1720110895.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2436769/photo1720110895.jpeg</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2816,7 +2816,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2710302/photo1756212500.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2710302/photo1756212500.jpeg</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2841,7 +2841,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2710301/photo1756212290.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2710301/photo1756212290.jpeg</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2438198/photo1720205449.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2438198/photo1720205449.jpeg.webp</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2886,7 +2886,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2710298/photo1756211718.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2710298/photo1756211718.jpeg</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2911,7 +2911,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2710296/photo1756210515.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2710296/photo1756210515.jpeg</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2936,7 +2936,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/1886202/200_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/1886202/200.webp</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2961,7 +2961,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2710903/photo1756347464.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2710903/photo1756347464.jpeg.webp</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2986,7 +2986,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2710902/photo1756346428.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2710902/photo1756346428.jpeg.webp</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -3011,7 +3011,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2710901/photo1756346231.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2710901/photo1756346231.jpeg.webp</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -3036,7 +3036,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2710900/photo1756346131.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2710900/photo1756346131.jpeg.webp</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3061,7 +3061,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2710899/photo1756345778.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2710899/photo1756345778.jpeg.webp</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3086,7 +3086,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2710898/photo1756345690.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2710898/photo1756345690.jpeg.webp</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3111,7 +3111,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2710897/photo1756345584.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2710897/photo1756345584.jpeg.webp</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3136,7 +3136,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2483470/photo1713999263.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2483470/photo1713999263.jpeg.webp</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3161,7 +3161,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2365057/photo1713999572.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2365057/photo1713999572.jpeg.webp</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3186,7 +3186,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>https://cdn.neemo.com.br/uploads/item/photo/2365056/photo1713999404.jpeg_item.png</t>
+          <t>https://cdn.neemo.com.br/uploads/item/photo/2365056/photo1713999404.jpeg.webp</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">

</xml_diff>